<commit_message>
Diss: Data Description Progress
</commit_message>
<xml_diff>
--- a/00_data/xx_column_mapping.xlsx
+++ b/00_data/xx_column_mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/29cb6aa242dd6fa3/00_Documents/06_university/00_university_of_sussex/05_summer_semester/05_dissertation/00_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morri\OneDrive\00_Documents\06_university\00_university_of_sussex\05_summer_semester\05_dissertation\00_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="8_{F140F6A3-C299-4B1C-A5CC-FBAEF598BA3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BE6935A-B48D-4DAB-B961-811244BD36C5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
   </bookViews>
   <sheets>
     <sheet name="xx_column_mapping" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
   <si>
     <t>Column Name</t>
   </si>
@@ -164,13 +164,124 @@
     <t>Y</t>
   </si>
   <si>
-    <t>datetime</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
     <t>date time separate columns</t>
+  </si>
+  <si>
+    <t>Column Explanation</t>
+  </si>
+  <si>
+    <t>String uniquely identifies the statement within the platform</t>
+  </si>
+  <si>
+    <t>category_specification_other</t>
+  </si>
+  <si>
+    <t>category_addition</t>
+  </si>
+  <si>
+    <t>category_specification</t>
+  </si>
+  <si>
+    <t>content_type</t>
+  </si>
+  <si>
+    <t>Type of content subject to restrictions - app, audio, image, product, synethetic (AI), text, video. Example: video modified by AI could be video and synthetic. Other can also be selected.</t>
+  </si>
+  <si>
+    <t>If 'other' is selected in 'content_type', a further specification is required.</t>
+  </si>
+  <si>
+    <t>Date of creation of the content i.e. when platform started hosting the information. Can be date that user was registered or date content posted.</t>
+  </si>
+  <si>
+    <t>Language of content. Either user account language or posted content language.</t>
+  </si>
+  <si>
+    <t>Visibility restrictions imposed on items i.e. content removal, disabling access, demotion, age restriction, interaction restriction or labelling.</t>
+  </si>
+  <si>
+    <t>Describes visabilitiy restriction that falls outside of categories in 'decision_visibility'.</t>
+  </si>
+  <si>
+    <t>Describes monetary payment restriction impost on information. Can be either 'suspension of monetary payments' or 'termination of monetary payments'.</t>
+  </si>
+  <si>
+    <t>Selected if a monetary decision does not fit into categories in 'decision_monetary'.</t>
+  </si>
+  <si>
+    <t>Restriction imposed on the provision of the service to a recipient of the service. Partial suspension, total suspension, partial termination or total termination.</t>
+  </si>
+  <si>
+    <t>Restriction imposed on the recipient of the service's account. Suspension or termination of the account.</t>
+  </si>
+  <si>
+    <t>Number/Character String</t>
+  </si>
+  <si>
+    <t>Blank = Indefinite, otherwise date</t>
+  </si>
+  <si>
+    <t>End date of visibility restriction</t>
+  </si>
+  <si>
+    <t>End date of monetary restriction</t>
+  </si>
+  <si>
+    <t>End date of service restriction</t>
+  </si>
+  <si>
+    <t>End date of account restriction</t>
+  </si>
+  <si>
+    <t>Source: https://transparency.dsa.ec.europa.eu/page/additional-explanation-for-statement-attributes</t>
+  </si>
+  <si>
+    <t>Data on Content Level</t>
+  </si>
+  <si>
+    <t>Date from which restrictions apply i.e. Start Date</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>String of 2 letter ISO code</t>
+  </si>
+  <si>
+    <t>[AT, BE, BG….]</t>
+  </si>
+  <si>
+    <t>Territorial scope of restrictions imposed. Can be EU &amp; EEA, EU or smaller group of countries.</t>
+  </si>
+  <si>
+    <t>Date Time</t>
+  </si>
+  <si>
+    <t>What led to the investigation of the content. Can be Article 16 (companies must make sure person or entity can report illegal content), notice from trsuted flagger or anything not under Article 16. Can also be voluntary from the platform. Orders from authorities not under Article 9 can be reported as 'other'.</t>
+  </si>
+  <si>
+    <t>Identity of notifier needs to be included in statement of reasons, but only if it is strictly necessary to identify the illegality of the content - for example in cases of infringements of intellectual property rights. Should not contain personal data.</t>
+  </si>
+  <si>
+    <t>Indicates whether the account holder is a business user under Regulation EU 2019/1150 or a private account for personal use only.</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>Yes, No</t>
+  </si>
+  <si>
+    <t>Were automated means used to identify specific content.</t>
+  </si>
+  <si>
+    <t>Fully automated, not automated, partially automated.</t>
+  </si>
+  <si>
+    <t>To what extent automated means were used to decide on infringing nature on the content. Refers to the decision not the identification of the content. Fully mean no human intervention, 'not' means entire decision by a human, 'partially means automated and human.</t>
   </si>
 </sst>
 </file>
@@ -195,10 +306,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Courier"/>
-      <family val="3"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -270,12 +383,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -291,9 +407,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,32 +743,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBEAE6A-8446-4184-AF47-49D8EAF8E74E}">
-  <dimension ref="B2:H37"/>
+  <dimension ref="B1:I41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="7" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="3" t="s">
+    <row r="1" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="G2" s="7"/>
       <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I2" s="8"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -664,210 +789,336 @@
         <v>38</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B25" t="s">
+      <c r="E28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
+      <c r="E29" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B27" t="s">
+      <c r="E30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B28" t="s">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B29" t="s">
+      <c r="C32" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" t="s">
+        <v>71</v>
+      </c>
+      <c r="E32" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B30" t="s">
+      <c r="C33" t="s">
+        <v>69</v>
+      </c>
+      <c r="E33" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B31" t="s">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B32" t="s">
+      <c r="E35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B33" t="s">
+      <c r="E36" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B34" t="s">
+      <c r="C37" t="s">
+        <v>77</v>
+      </c>
+      <c r="D37" t="s">
+        <v>78</v>
+      </c>
+      <c r="E37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
+      <c r="C38" t="s">
+        <v>77</v>
+      </c>
+      <c r="D38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E38" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B36" t="s">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B37" t="s">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
         <v>35</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C41" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" s="9">
+        <v>46071.40525462963</v>
+      </c>
+      <c r="E41" s="9"/>
+      <c r="F41" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D37" s="8">
-        <v>46071.40525462963</v>
-      </c>
-      <c r="E37" s="1" t="s">
+      <c r="G41" t="s">
+        <v>39</v>
+      </c>
+      <c r="H41" t="s">
         <v>43</v>
-      </c>
-      <c r="F37" t="s">
-        <v>39</v>
-      </c>
-      <c r="G37" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="F2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Diss: Cleaning - Territory Fix & Aggregation Progress
</commit_message>
<xml_diff>
--- a/00_data/xx_column_mapping.xlsx
+++ b/00_data/xx_column_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/29cb6aa242dd6fa3/00_Documents/06_university/00_university_of_sussex/05_summer_semester/05_dissertation/00_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="614" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BCA2924-3421-4706-9AE4-80048FFA76B0}"/>
+  <xr:revisionPtr revIDLastSave="665" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35A8B44A-26FC-4CEC-8AA3-1FF06E90196A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="215">
   <si>
     <t>Column Name</t>
   </si>
@@ -612,6 +612,75 @@
   </si>
   <si>
     <t>cont_lang</t>
+  </si>
+  <si>
+    <t>Column Description</t>
+  </si>
+  <si>
+    <t>Territory</t>
+  </si>
+  <si>
+    <t>Date of SOR</t>
+  </si>
+  <si>
+    <t>Time of SOR</t>
+  </si>
+  <si>
+    <t>Content Created Date</t>
+  </si>
+  <si>
+    <t>Date of Restriction Applied</t>
+  </si>
+  <si>
+    <t>Automated Detection</t>
+  </si>
+  <si>
+    <t>Automated Decision</t>
+  </si>
+  <si>
+    <t>Content Language</t>
+  </si>
+  <si>
+    <t>Content Type</t>
+  </si>
+  <si>
+    <t>Source Type - How was content found</t>
+  </si>
+  <si>
+    <t>Content Category - High Level</t>
+  </si>
+  <si>
+    <t>Content Category - More Detail</t>
+  </si>
+  <si>
+    <t>Context for Decision</t>
+  </si>
+  <si>
+    <t>Context if content was illegal</t>
+  </si>
+  <si>
+    <t>Decision on content - was content removed, disabled, age restricted etc.</t>
+  </si>
+  <si>
+    <t>Describes restriction outside des_vis scope</t>
+  </si>
+  <si>
+    <t>Date restriction ended</t>
+  </si>
+  <si>
+    <t>Decision on monetary restriction on account</t>
+  </si>
+  <si>
+    <t>Describes what happened to account outside of des_mon scope</t>
+  </si>
+  <si>
+    <t>Describes whether services were suspended or terminated to a customer</t>
+  </si>
+  <si>
+    <t>Describes account decision - suspended or terminated</t>
+  </si>
+  <si>
+    <t>Decision Ground - Was the content illegal or against terms and conditions?</t>
   </si>
 </sst>
 </file>
@@ -668,7 +737,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -793,11 +862,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -865,6 +986,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -883,44 +1034,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1265,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBEAE6A-8446-4184-AF47-49D8EAF8E74E}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -1283,9 +1406,10 @@
     <col min="13" max="13" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="25.21875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="67.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>145</v>
       </c>
@@ -1308,28 +1432,29 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="23" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="25"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="34"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="35"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>75</v>
       </c>
@@ -1360,7 +1485,7 @@
       <c r="J3" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="30" t="s">
         <v>188</v>
       </c>
       <c r="L3" s="4" t="s">
@@ -1375,8 +1500,11 @@
       <c r="O3" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P3" s="39" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>36</v>
       </c>
@@ -1401,13 +1529,13 @@
       <c r="H4" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="33" t="s">
+      <c r="I4" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4" s="25" t="s">
         <v>39</v>
       </c>
       <c r="L4" s="8">
@@ -1419,11 +1547,14 @@
       <c r="N4" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="O4" s="36" t="s">
+      <c r="O4" s="28" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P4" s="40" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>29</v>
       </c>
@@ -1445,77 +1576,83 @@
       <c r="G5" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H5" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L5" s="31">
+      <c r="H5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" s="10">
         <v>2</v>
       </c>
-      <c r="M5" s="29" t="s">
+      <c r="M5" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="N5" s="29" t="s">
+      <c r="N5" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O5" s="11" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P5" s="41" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>38</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="30">
+      <c r="D6" s="23">
         <v>46071.40525462963</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="F6" s="30"/>
+      <c r="F6" s="23"/>
       <c r="G6" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H6" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="J6" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K6" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L6" s="31">
+      <c r="H6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K6" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="10">
         <v>3</v>
       </c>
-      <c r="M6" s="29" t="s">
+      <c r="M6" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="N6" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O6" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P6" s="42" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1525,32 +1662,35 @@
       <c r="G7" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H7" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="J7" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L7" s="31">
+      <c r="H7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L7" s="10">
         <v>4</v>
       </c>
-      <c r="M7" s="29" t="s">
+      <c r="M7" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="N7" s="29" t="s">
+      <c r="N7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="O7" s="34">
+      <c r="O7" s="26">
         <v>0.6875</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P7" s="42" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>27</v>
       </c>
@@ -1572,32 +1712,35 @@
       <c r="G8" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H8" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K8" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L8" s="31">
+      <c r="H8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" s="10">
         <v>5</v>
       </c>
-      <c r="M8" s="29" t="s">
+      <c r="M8" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="N8" s="29" t="s">
+      <c r="N8" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O8" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P8" s="42" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>30</v>
       </c>
@@ -1619,30 +1762,33 @@
       <c r="G9" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H9" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K9" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L9" s="31">
+      <c r="H9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" s="10">
         <v>6</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="M9" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="N9" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O9" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P9" s="42" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>34</v>
       </c>
@@ -1664,30 +1810,33 @@
       <c r="G10" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="31"/>
-      <c r="J10" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K10" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L10" s="31">
+      <c r="H10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="10"/>
+      <c r="J10" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K10" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L10" s="10">
         <v>7</v>
       </c>
-      <c r="M10" s="29" t="s">
+      <c r="M10" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="N10" s="29" t="s">
+      <c r="N10" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O10" s="11" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P10" s="41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>35</v>
       </c>
@@ -1709,30 +1858,33 @@
       <c r="G11" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H11" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="31"/>
-      <c r="J11" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K11" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L11" s="31">
+      <c r="H11" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I11" s="10"/>
+      <c r="J11" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K11" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L11" s="10">
         <v>8</v>
       </c>
-      <c r="M11" s="29" t="s">
+      <c r="M11" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="29" t="s">
+      <c r="N11" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O11" s="11" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P11" s="41" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>24</v>
       </c>
@@ -1754,30 +1906,33 @@
       <c r="G12" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H12" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12" s="31"/>
-      <c r="J12" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K12" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L12" s="31">
+      <c r="H12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" s="10"/>
+      <c r="J12" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K12" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L12" s="10">
         <v>9</v>
       </c>
-      <c r="M12" s="29" t="s">
+      <c r="M12" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="N12" s="29" t="s">
+      <c r="N12" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O12" s="11" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P12" s="41" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>26</v>
       </c>
@@ -1799,30 +1954,33 @@
       <c r="G13" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H13" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K13" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L13" s="31">
+      <c r="H13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K13" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L13" s="10">
         <v>10</v>
       </c>
-      <c r="M13" s="29" t="s">
+      <c r="M13" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="N13" s="29" t="s">
+      <c r="N13" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O13" s="11" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P13" s="41" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>32</v>
       </c>
@@ -1844,30 +2002,33 @@
       <c r="G14" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H14" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I14" s="31"/>
-      <c r="J14" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L14" s="31">
+      <c r="H14" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K14" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L14" s="10">
         <v>11</v>
       </c>
-      <c r="M14" s="29" t="s">
+      <c r="M14" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="N14" s="29" t="s">
+      <c r="N14" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O14" s="11" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P14" s="41" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>20</v>
       </c>
@@ -1889,30 +2050,33 @@
       <c r="G15" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H15" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I15" s="31"/>
-      <c r="J15" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K15" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L15" s="31">
+      <c r="H15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I15" s="10"/>
+      <c r="J15" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K15" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="10">
         <v>12</v>
       </c>
-      <c r="M15" s="29" t="s">
+      <c r="M15" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="N15" s="29" t="s">
+      <c r="N15" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O15" s="11" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P15" s="41" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>22</v>
       </c>
@@ -1934,30 +2098,33 @@
       <c r="G16" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I16" s="31"/>
-      <c r="J16" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K16" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L16" s="31">
+      <c r="H16" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I16" s="10"/>
+      <c r="J16" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K16" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L16" s="10">
         <v>13</v>
       </c>
-      <c r="M16" s="29" t="s">
+      <c r="M16" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="N16" s="29" t="s">
+      <c r="N16" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O16" s="11" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P16" s="41" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>13</v>
       </c>
@@ -1979,30 +2146,33 @@
       <c r="G17" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H17" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I17" s="31"/>
-      <c r="J17" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K17" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L17" s="31">
+      <c r="H17" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I17" s="10"/>
+      <c r="J17" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K17" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L17" s="10">
         <v>14</v>
       </c>
-      <c r="M17" s="29" t="s">
+      <c r="M17" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="N17" s="29" t="s">
+      <c r="N17" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O17" s="11" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P17" s="41" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -2024,30 +2194,33 @@
       <c r="G18" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H18" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I18" s="31"/>
-      <c r="J18" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K18" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L18" s="31">
+      <c r="H18" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K18" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L18" s="10">
         <v>15</v>
       </c>
-      <c r="M18" s="29" t="s">
+      <c r="M18" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="N18" s="29" t="s">
+      <c r="N18" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O18" s="11" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P18" s="41" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>19</v>
       </c>
@@ -2069,30 +2242,33 @@
       <c r="G19" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H19" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K19" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L19" s="31">
+      <c r="H19" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K19" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L19" s="10">
         <v>16</v>
       </c>
-      <c r="M19" s="29" t="s">
+      <c r="M19" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="N19" s="29" t="s">
+      <c r="N19" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O19" s="11" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P19" s="41" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
         <v>2</v>
       </c>
@@ -2114,30 +2290,33 @@
       <c r="G20" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H20" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I20" s="31"/>
-      <c r="J20" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K20" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L20" s="31">
+      <c r="H20" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K20" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L20" s="10">
         <v>17</v>
       </c>
-      <c r="M20" s="29" t="s">
+      <c r="M20" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="N20" s="29" t="s">
+      <c r="N20" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O20" s="11" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P20" s="41" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>3</v>
       </c>
@@ -2159,30 +2338,33 @@
       <c r="G21" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H21" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I21" s="31"/>
-      <c r="J21" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K21" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L21" s="31">
+      <c r="H21" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K21" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L21" s="10">
         <v>18</v>
       </c>
-      <c r="M21" s="29" t="s">
+      <c r="M21" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="N21" s="29" t="s">
+      <c r="N21" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O21" s="11" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P21" s="41" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>4</v>
       </c>
@@ -2204,30 +2386,33 @@
       <c r="G22" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H22" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I22" s="31"/>
-      <c r="J22" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K22" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L22" s="31">
+      <c r="H22" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K22" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L22" s="10">
         <v>19</v>
       </c>
-      <c r="M22" s="29" t="s">
+      <c r="M22" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="N22" s="29" t="s">
+      <c r="N22" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O22" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P22" s="41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>5</v>
       </c>
@@ -2249,30 +2434,33 @@
       <c r="G23" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H23" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I23" s="31"/>
-      <c r="J23" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K23" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L23" s="31">
+      <c r="H23" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I23" s="10"/>
+      <c r="J23" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K23" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L23" s="10">
         <v>20</v>
       </c>
-      <c r="M23" s="29" t="s">
+      <c r="M23" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="N23" s="29" t="s">
+      <c r="N23" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O23" s="11" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P23" s="41" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>6</v>
       </c>
@@ -2294,30 +2482,33 @@
       <c r="G24" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H24" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K24" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L24" s="31">
+      <c r="H24" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K24" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L24" s="10">
         <v>21</v>
       </c>
-      <c r="M24" s="29" t="s">
+      <c r="M24" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="N24" s="29" t="s">
+      <c r="N24" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O24" s="11" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P24" s="41" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>7</v>
       </c>
@@ -2339,30 +2530,33 @@
       <c r="G25" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H25" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I25" s="31"/>
-      <c r="J25" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K25" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L25" s="31">
+      <c r="H25" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L25" s="10">
         <v>22</v>
       </c>
-      <c r="M25" s="29" t="s">
+      <c r="M25" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="N25" s="29" t="s">
+      <c r="N25" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O25" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P25" s="41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
         <v>8</v>
       </c>
@@ -2384,30 +2578,33 @@
       <c r="G26" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H26" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I26" s="31"/>
-      <c r="J26" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K26" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L26" s="31">
+      <c r="H26" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I26" s="10"/>
+      <c r="J26" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K26" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L26" s="10">
         <v>23</v>
       </c>
-      <c r="M26" s="29" t="s">
+      <c r="M26" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="N26" s="29" t="s">
+      <c r="N26" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O26" s="11" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P26" s="41" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>9</v>
       </c>
@@ -2429,30 +2626,33 @@
       <c r="G27" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H27" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K27" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L27" s="31">
+      <c r="H27" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K27" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L27" s="10">
         <v>24</v>
       </c>
-      <c r="M27" s="29" t="s">
+      <c r="M27" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="N27" s="29" t="s">
+      <c r="N27" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O27" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P27" s="41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
         <v>10</v>
       </c>
@@ -2474,28 +2674,31 @@
       <c r="G28" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H28" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I28" s="31"/>
-      <c r="J28" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K28" s="38"/>
-      <c r="L28" s="31">
+      <c r="H28" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I28" s="10"/>
+      <c r="J28" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10">
         <v>25</v>
       </c>
-      <c r="M28" s="29" t="s">
+      <c r="M28" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="N28" s="29" t="s">
+      <c r="N28" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O28" s="11" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P28" s="41" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="9">
         <v>11</v>
       </c>
@@ -2517,75 +2720,81 @@
       <c r="G29" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H29" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I29" s="31"/>
-      <c r="J29" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K29" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="L29" s="31">
+      <c r="H29" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K29" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L29" s="10">
         <v>26</v>
       </c>
-      <c r="M29" s="29" t="s">
+      <c r="M29" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="N29" s="29" t="s">
+      <c r="N29" s="1" t="s">
         <v>64</v>
       </c>
       <c r="O29" s="21">
         <v>46055</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P29" s="41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
         <v>1</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="E30" s="31" t="s">
+      <c r="E30" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="F30" s="29" t="s">
+      <c r="F30" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G30" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H30" s="31" t="s">
+      <c r="H30" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I30" s="31"/>
-      <c r="J30" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K30" s="40" t="s">
+      <c r="I30" s="10"/>
+      <c r="J30" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K30" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L30" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M30" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N30" s="29" t="s">
+      <c r="L30" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N30" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O30" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P30" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="9">
         <v>12</v>
       </c>
@@ -2607,30 +2816,33 @@
       <c r="G31" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H31" s="31" t="s">
+      <c r="H31" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K31" s="40" t="s">
+      <c r="I31" s="10"/>
+      <c r="J31" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K31" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L31" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M31" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N31" s="29" t="s">
+      <c r="L31" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N31" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O31" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P31" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="9">
         <v>14</v>
       </c>
@@ -2652,30 +2864,33 @@
       <c r="G32" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H32" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I32" s="31"/>
-      <c r="J32" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K32" s="40" t="s">
+      <c r="H32" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K32" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L32" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M32" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N32" s="29" t="s">
+      <c r="L32" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N32" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O32" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P32" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="9">
         <v>15</v>
       </c>
@@ -2697,30 +2912,33 @@
       <c r="G33" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H33" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I33" s="31"/>
-      <c r="J33" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K33" s="40" t="s">
+      <c r="H33" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K33" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L33" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M33" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N33" s="29" t="s">
+      <c r="L33" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N33" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O33" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P33" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="9">
         <v>16</v>
       </c>
@@ -2742,30 +2960,33 @@
       <c r="G34" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H34" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K34" s="40" t="s">
+      <c r="H34" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K34" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L34" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M34" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N34" s="29" t="s">
+      <c r="L34" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N34" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O34" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P34" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="9">
         <v>18</v>
       </c>
@@ -2785,30 +3006,33 @@
       <c r="G35" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H35" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K35" s="40" t="s">
+      <c r="H35" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K35" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L35" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M35" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N35" s="29" t="s">
+      <c r="L35" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N35" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O35" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P35" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="9">
         <v>21</v>
       </c>
@@ -2830,30 +3054,33 @@
       <c r="G36" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H36" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I36" s="31"/>
-      <c r="J36" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K36" s="40" t="s">
+      <c r="H36" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K36" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L36" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M36" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N36" s="29" t="s">
+      <c r="L36" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N36" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O36" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P36" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="9">
         <v>23</v>
       </c>
@@ -2875,30 +3102,33 @@
       <c r="G37" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H37" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I37" s="31"/>
-      <c r="J37" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K37" s="40" t="s">
+      <c r="H37" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K37" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L37" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M37" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N37" s="29" t="s">
+      <c r="L37" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N37" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O37" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P37" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="9">
         <v>25</v>
       </c>
@@ -2920,30 +3150,33 @@
       <c r="G38" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H38" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K38" s="40" t="s">
+      <c r="H38" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K38" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L38" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M38" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N38" s="29" t="s">
+      <c r="L38" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N38" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O38" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P38" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
         <v>28</v>
       </c>
@@ -2965,30 +3198,33 @@
       <c r="G39" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H39" s="31" t="s">
+      <c r="H39" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I39" s="31"/>
-      <c r="J39" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K39" s="40" t="s">
+      <c r="I39" s="10"/>
+      <c r="J39" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K39" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L39" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M39" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N39" s="29" t="s">
+      <c r="L39" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N39" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O39" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P39" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="9">
         <v>31</v>
       </c>
@@ -3010,30 +3246,33 @@
       <c r="G40" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H40" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I40" s="31"/>
-      <c r="J40" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K40" s="40" t="s">
+      <c r="H40" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K40" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L40" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M40" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N40" s="29" t="s">
+      <c r="L40" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N40" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O40" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P40" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="16">
         <v>33</v>
       </c>
@@ -3055,31 +3294,34 @@
       <c r="G41" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="H41" s="31" t="s">
+      <c r="H41" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I41" s="31"/>
-      <c r="J41" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="K41" s="40" t="s">
+      <c r="I41" s="10"/>
+      <c r="J41" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="K41" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="L41" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="M41" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="N41" s="29" t="s">
+      <c r="L41" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N41" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O41" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="29">
+      <c r="P41" s="41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
         <v>37</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -3107,7 +3349,7 @@
       <c r="J42" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="K42" s="41" t="s">
+      <c r="K42" s="32" t="s">
         <v>40</v>
       </c>
       <c r="L42" s="18" t="s">
@@ -3119,7 +3361,10 @@
       <c r="N42" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="O42" s="35" t="s">
+      <c r="O42" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="P42" s="43" t="s">
         <v>148</v>
       </c>
     </row>
@@ -3128,8 +3373,8 @@
     <sortCondition ref="L4:L42"/>
   </sortState>
   <mergeCells count="2">
-    <mergeCell ref="G2:O2"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="G2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Diss: Initial Data Visualisation
</commit_message>
<xml_diff>
--- a/00_data/xx_column_mapping.xlsx
+++ b/00_data/xx_column_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/29cb6aa242dd6fa3/00_Documents/06_university/00_university_of_sussex/05_summer_semester/05_dissertation/00_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="847" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F10963-6844-452A-A0CE-571D1163F32B}"/>
+  <xr:revisionPtr revIDLastSave="853" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7802705-95DD-4D2D-BDB6-7B12640B80D0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
   </bookViews>
   <sheets>
     <sheet name="xx_column_mapping" sheetId="1" r:id="rId1"/>
@@ -917,7 +917,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -970,77 +970,71 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1061,10 +1055,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1391,8 +1381,8 @@
     <col min="2" max="2" width="31.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" customWidth="1"/>
     <col min="4" max="4" width="43.77734375" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" customWidth="1"/>
-    <col min="6" max="6" width="21.88671875" customWidth="1"/>
+    <col min="5" max="5" width="66.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5546875" customWidth="1"/>
     <col min="8" max="8" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="30.5546875" customWidth="1"/>
@@ -1430,27 +1420,27 @@
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="28" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1501,173 +1491,181 @@
       <c r="P3" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="Q3" s="42" t="s">
+      <c r="Q3" s="27" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
-        <v>36</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="E4" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="33" t="s">
-        <v>96</v>
+      <c r="F4" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="H4" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4" s="34">
-        <v>1</v>
-      </c>
-      <c r="M4" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="N4" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="O4" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="P4" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q4" s="38" t="s">
-        <v>39</v>
+        <v>140</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="P4" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q4" s="23" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="18">
-        <v>46071.40525462963</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="F5" s="18"/>
+        <v>71</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="G5" s="15" t="s">
         <v>141</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K5" s="22" t="s">
+      <c r="I5" s="6"/>
+      <c r="J5" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L5" s="6">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O5" s="16">
-        <v>46055</v>
-      </c>
-      <c r="P5" s="37" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q5" s="40" t="s">
+        <v>71</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q5" s="25" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="A6" s="5">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>52</v>
+      </c>
       <c r="G6" s="15" t="s">
         <v>141</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="I6" s="6"/>
       <c r="J6" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K6" s="22" t="s">
+      <c r="K6" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L6" s="6">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="O6" s="20">
-        <v>0.6875</v>
-      </c>
-      <c r="P6" s="37" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q6" s="40" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q6" s="25" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="10">
-        <v>46041</v>
-      </c>
-      <c r="E7" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>118</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>141</v>
@@ -1675,20 +1673,18 @@
       <c r="H7" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="I7" s="6"/>
       <c r="J7" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="K7" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L7" s="6">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>64</v>
@@ -1696,31 +1692,31 @@
       <c r="O7" s="16">
         <v>46055</v>
       </c>
-      <c r="P7" s="37" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q7" s="40" t="s">
-        <v>39</v>
+      <c r="P7" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q7" s="25" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="10">
-        <v>45789</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>118</v>
+        <v>71</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>141</v>
@@ -1729,49 +1725,49 @@
         <v>39</v>
       </c>
       <c r="I8" s="6"/>
-      <c r="J8" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K8" s="22" t="s">
+      <c r="J8" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K8" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L8" s="6">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O8" s="16">
-        <v>46055</v>
-      </c>
-      <c r="P8" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q8" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="P8" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q8" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>114</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>141</v>
@@ -1780,49 +1776,49 @@
         <v>39</v>
       </c>
       <c r="I9" s="6"/>
-      <c r="J9" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K9" s="22" t="s">
+      <c r="J9" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K9" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L9" s="6">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="P9" s="25" t="s">
-        <v>196</v>
-      </c>
-      <c r="Q9" s="39" t="s">
-        <v>39</v>
+        <v>179</v>
+      </c>
+      <c r="P9" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q9" s="24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>118</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>141</v>
@@ -1831,49 +1827,49 @@
         <v>39</v>
       </c>
       <c r="I10" s="6"/>
-      <c r="J10" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K10" s="22" t="s">
+      <c r="J10" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K10" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L10" s="6">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="P10" s="25" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q10" s="39" t="s">
-        <v>39</v>
+        <v>64</v>
+      </c>
+      <c r="O10" s="16">
+        <v>46055</v>
+      </c>
+      <c r="P10" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q10" s="24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>141</v>
@@ -1882,49 +1878,49 @@
         <v>39</v>
       </c>
       <c r="I11" s="6"/>
-      <c r="J11" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K11" s="22" t="s">
+      <c r="J11" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K11" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L11" s="6">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>189</v>
+        <v>167</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="P11" s="25" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q11" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="P11" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q11" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>137</v>
+        <v>58</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>136</v>
+        <v>82</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>141</v>
@@ -1936,46 +1932,46 @@
       <c r="J12" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K12" s="22" t="s">
+      <c r="K12" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L12" s="6">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="O12" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="P12" s="25" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q12" s="39" t="s">
-        <v>39</v>
+        <v>64</v>
+      </c>
+      <c r="O12" s="16">
+        <v>46055</v>
+      </c>
+      <c r="P12" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q12" s="24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="G13" s="15" t="s">
         <v>141</v>
@@ -1984,49 +1980,49 @@
         <v>39</v>
       </c>
       <c r="I13" s="6"/>
-      <c r="J13" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K13" s="22" t="s">
+      <c r="J13" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K13" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L13" s="6">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="P13" s="25" t="s">
-        <v>200</v>
-      </c>
-      <c r="Q13" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="P13" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q13" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>118</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="G14" s="15" t="s">
         <v>141</v>
@@ -2035,202 +2031,202 @@
         <v>39</v>
       </c>
       <c r="I14" s="6"/>
-      <c r="J14" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="22" t="s">
+      <c r="J14" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K14" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L14" s="6">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="O14" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="P14" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q14" s="39" t="s">
-        <v>39</v>
+        <v>64</v>
+      </c>
+      <c r="O14" s="16">
+        <v>46055</v>
+      </c>
+      <c r="P14" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q14" s="24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>119</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I15" s="6"/>
-      <c r="J15" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K15" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L15" s="6">
-        <v>12</v>
+      <c r="J15" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K15" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="P15" s="25" t="s">
-        <v>202</v>
-      </c>
-      <c r="Q15" s="39" t="s">
-        <v>39</v>
+        <v>148</v>
+      </c>
+      <c r="P15" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q15" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>39</v>
       </c>
       <c r="I16" s="6"/>
-      <c r="J16" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K16" s="22" t="s">
+      <c r="J16" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K16" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L16" s="6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>216</v>
+        <v>158</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>220</v>
+        <v>71</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="P16" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q16" s="39" t="s">
-        <v>40</v>
+        <v>178</v>
+      </c>
+      <c r="P16" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q16" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>39</v>
       </c>
       <c r="I17" s="6"/>
-      <c r="J17" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K17" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L17" s="6">
-        <v>14</v>
+      <c r="J17" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K17" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="P17" s="25" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q17" s="39" t="s">
-        <v>39</v>
+        <v>148</v>
+      </c>
+      <c r="P17" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q17" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="G18" s="15" t="s">
         <v>140</v>
@@ -2242,14 +2238,14 @@
       <c r="J18" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K18" s="22" t="s">
+      <c r="K18" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L18" s="6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N18" s="1" t="s">
         <v>220</v>
@@ -2257,31 +2253,31 @@
       <c r="O18" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="P18" s="25" t="s">
+      <c r="P18" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="Q18" s="39" t="s">
+      <c r="Q18" s="24" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G19" s="15" t="s">
         <v>140</v>
@@ -2293,14 +2289,14 @@
       <c r="J19" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K19" s="22" t="s">
+      <c r="K19" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L19" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>220</v>
@@ -2308,34 +2304,34 @@
       <c r="O19" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="P19" s="25" t="s">
+      <c r="P19" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="Q19" s="39" t="s">
+      <c r="Q19" s="24" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>128</v>
+        <v>71</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>129</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>39</v>
@@ -2344,14 +2340,14 @@
       <c r="J20" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K20" s="22" t="s">
+      <c r="K20" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L20" s="6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>220</v>
@@ -2359,34 +2355,32 @@
       <c r="O20" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="P20" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q20" s="39" t="s">
+      <c r="P20" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q20" s="24" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>129</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="6"/>
       <c r="F21" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>39</v>
@@ -2395,26 +2389,26 @@
       <c r="J21" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K21" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L21" s="6">
-        <v>18</v>
+      <c r="K21" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>220</v>
+        <v>148</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="P21" s="25" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q21" s="39" t="s">
-        <v>40</v>
+        <v>148</v>
+      </c>
+      <c r="P21" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q21" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -2446,7 +2440,7 @@
       <c r="J22" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K22" s="22" t="s">
+      <c r="K22" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L22" s="6">
@@ -2461,31 +2455,31 @@
       <c r="O22" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="P22" s="25" t="s">
+      <c r="P22" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="Q22" s="39" t="s">
+      <c r="Q22" s="24" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="G23" s="15" t="s">
         <v>141</v>
@@ -2494,52 +2488,52 @@
         <v>39</v>
       </c>
       <c r="I23" s="6"/>
-      <c r="J23" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K23" s="22" t="s">
+      <c r="J23" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K23" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L23" s="6">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="P23" s="25" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q23" s="39" t="s">
+        <v>176</v>
+      </c>
+      <c r="P23" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q23" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>39</v>
@@ -2548,46 +2542,46 @@
       <c r="J24" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K24" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L24" s="6">
-        <v>21</v>
+      <c r="K24" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="O24" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="P24" s="25" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q24" s="39" t="s">
-        <v>40</v>
+        <v>148</v>
+      </c>
+      <c r="P24" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q24" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>59</v>
+        <v>106</v>
       </c>
       <c r="G25" s="15" t="s">
         <v>141</v>
@@ -2596,100 +2590,100 @@
         <v>39</v>
       </c>
       <c r="I25" s="6"/>
-      <c r="J25" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K25" s="22" t="s">
+      <c r="J25" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K25" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L25" s="6">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O25" s="16">
-        <v>46055</v>
-      </c>
-      <c r="P25" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q25" s="39" t="s">
-        <v>40</v>
+        <v>71</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="P25" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q25" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>71</v>
+        <v>130</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>39</v>
       </c>
       <c r="I26" s="6"/>
-      <c r="J26" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K26" s="22" t="s">
+      <c r="J26" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K26" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L26" s="6">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>164</v>
+        <v>216</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>71</v>
+        <v>220</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="P26" s="25" t="s">
-        <v>208</v>
-      </c>
-      <c r="Q26" s="39" t="s">
-        <v>39</v>
+        <v>221</v>
+      </c>
+      <c r="P26" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q26" s="24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="G27" s="15" t="s">
         <v>141</v>
@@ -2698,52 +2692,52 @@
         <v>39</v>
       </c>
       <c r="I27" s="6"/>
-      <c r="J27" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K27" s="22" t="s">
+      <c r="J27" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K27" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L27" s="6">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="P27" s="25" t="s">
-        <v>209</v>
-      </c>
-      <c r="Q27" s="39" t="s">
-        <v>40</v>
+        <v>174</v>
+      </c>
+      <c r="P27" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q27" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>58</v>
+        <v>130</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>39</v>
@@ -2752,46 +2746,46 @@
       <c r="J28" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K28" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L28" s="6">
-        <v>25</v>
+      <c r="K28" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O28" s="16">
-        <v>46055</v>
-      </c>
-      <c r="P28" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q28" s="39" t="s">
-        <v>40</v>
+        <v>148</v>
+      </c>
+      <c r="O28" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="P28" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q28" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G29" s="15" t="s">
         <v>141</v>
@@ -2800,49 +2794,49 @@
         <v>39</v>
       </c>
       <c r="I29" s="6"/>
-      <c r="J29" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K29" s="22" t="s">
+      <c r="J29" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K29" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L29" s="6">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="N29" s="1" t="s">
         <v>71</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="P29" s="25" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q29" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="P29" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q29" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" s="5">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E30" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="10">
+        <v>46041</v>
+      </c>
+      <c r="E30" s="11" t="s">
         <v>118</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="G30" s="15" t="s">
         <v>141</v>
@@ -2850,18 +2844,20 @@
       <c r="H30" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I30" s="6"/>
+      <c r="I30" s="18" t="s">
+        <v>39</v>
+      </c>
       <c r="J30" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K30" s="22" t="s">
+      <c r="K30" s="18" t="s">
         <v>39</v>
       </c>
       <c r="L30" s="6">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="N30" s="1" t="s">
         <v>64</v>
@@ -2869,82 +2865,82 @@
       <c r="O30" s="16">
         <v>46055</v>
       </c>
-      <c r="P30" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q30" s="39" t="s">
-        <v>40</v>
+      <c r="P30" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q30" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" s="5">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I31" s="6"/>
-      <c r="J31" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K31" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L31" s="6">
-        <v>28</v>
+      <c r="J31" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K31" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>148</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="O31" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="P31" s="25" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q31" s="39" t="s">
-        <v>39</v>
+        <v>148</v>
+      </c>
+      <c r="P31" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q31" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" s="5">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>118</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G32" s="15" t="s">
         <v>141</v>
@@ -2952,50 +2948,52 @@
       <c r="H32" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K32" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L32" s="6">
-        <v>29</v>
+      <c r="I32" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="J32" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>217</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O32" s="16">
-        <v>46055</v>
-      </c>
-      <c r="P32" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q32" s="39" t="s">
-        <v>40</v>
+        <v>220</v>
+      </c>
+      <c r="O32" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="P32" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q32" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E33" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="10">
+        <v>45789</v>
+      </c>
+      <c r="E33" s="11" t="s">
         <v>118</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G33" s="15" t="s">
         <v>141</v>
@@ -3003,166 +3001,164 @@
       <c r="H33" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I33" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="J33" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K33" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>217</v>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K33" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L33" s="6">
+        <v>5</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="O33" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="P33" s="25" t="s">
-        <v>218</v>
-      </c>
-      <c r="Q33" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="O33" s="16">
+        <v>46055</v>
+      </c>
+      <c r="P33" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q33" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="5">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>57</v>
+        <v>143</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>118</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="G34" s="15" t="s">
         <v>140</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K34" s="23" t="s">
+      <c r="K34" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L34" s="6">
+        <v>15</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="O34" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="P34" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q34" s="24" t="s">
         <v>40</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="M34" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="O34" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P34" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q34" s="39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="5">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I35" s="6"/>
-      <c r="J35" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K35" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>148</v>
+      <c r="J35" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L35" s="6">
+        <v>10</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>148</v>
+        <v>71</v>
       </c>
       <c r="O35" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P35" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q35" s="39" t="s">
-        <v>148</v>
+        <v>173</v>
+      </c>
+      <c r="P35" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="Q35" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
-        <v>14</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E36" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="D36" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="E36" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>84</v>
+      <c r="F36" s="33" t="s">
+        <v>90</v>
       </c>
       <c r="G36" s="15" t="s">
         <v>140</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="K36" s="23" t="s">
+      <c r="K36" s="19" t="s">
         <v>40</v>
       </c>
       <c r="L36" s="6" t="s">
@@ -3177,320 +3173,314 @@
       <c r="O36" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="P36" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q36" s="39" t="s">
+      <c r="P36" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q36" s="24" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="5">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E37" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>118</v>
+      </c>
       <c r="F37" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>39</v>
       </c>
       <c r="I37" s="6"/>
-      <c r="J37" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K37" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>148</v>
+      <c r="J37" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K37" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L37" s="6">
+        <v>6</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>148</v>
+        <v>71</v>
       </c>
       <c r="O37" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P37" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q37" s="39" t="s">
-        <v>148</v>
+        <v>171</v>
+      </c>
+      <c r="P37" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q37" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>39</v>
       </c>
       <c r="I38" s="6"/>
-      <c r="J38" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K38" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="L38" s="6" t="s">
-        <v>148</v>
+      <c r="J38" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K38" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L38" s="6">
+        <v>7</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>148</v>
+        <v>71</v>
       </c>
       <c r="O38" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P38" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q38" s="39" t="s">
-        <v>148</v>
+        <v>172</v>
+      </c>
+      <c r="P38" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q38" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" s="5">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K39" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>148</v>
+      <c r="I39" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="J39" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="K39" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L39" s="6">
+        <v>1</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="O39" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P39" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q39" s="39" t="s">
-        <v>148</v>
+        <v>71</v>
+      </c>
+      <c r="O39" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="P39" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q39" s="24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="G40" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H40" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K40" s="23" t="s">
+      <c r="I40" s="35"/>
+      <c r="J40" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="K40" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="L40" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="M40" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="N40" s="1" t="s">
+      <c r="L40" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="M40" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="N40" s="33" t="s">
         <v>148</v>
       </c>
       <c r="O40" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="P40" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q40" s="39" t="s">
+      <c r="P40" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q40" s="24" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="12">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="D41" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="F41" s="13" t="s">
-        <v>90</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="D41" s="34">
+        <v>46071.40525462963</v>
+      </c>
+      <c r="E41" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" s="34"/>
       <c r="G41" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H41" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I41" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K41" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="L41" s="6">
+        <v>2</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="O41" s="16">
+        <v>46055</v>
+      </c>
+      <c r="P41" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q41" s="24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A42" s="33"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I42" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="J42" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="K42" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="L42" s="14">
+        <v>3</v>
+      </c>
+      <c r="M42" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="N42" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="O42" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="P42" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q42" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K41" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="M41" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="N41" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="O41" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="P41" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q41" s="39" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
-        <v>37</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G42" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="H42" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="K42" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="L42" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="M42" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="N42" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="O42" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="P42" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q42" s="41" t="s">
-        <v>148</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:P42">
-    <sortCondition ref="L4:L42"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:Q42">
+    <sortCondition ref="A4:A42"/>
   </sortState>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Diss: Pipeline Scale Up - RQs
</commit_message>
<xml_diff>
--- a/00_data/xx_column_mapping.xlsx
+++ b/00_data/xx_column_mapping.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="853" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7802705-95DD-4D2D-BDB6-7B12640B80D0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
   </bookViews>
   <sheets>
     <sheet name="xx_column_mapping" sheetId="1" r:id="rId1"/>
@@ -917,7 +917,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -998,6 +998,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1013,28 +1026,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1055,6 +1046,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1420,27 +1415,27 @@
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31" t="s">
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -3133,19 +3128,19 @@
       <c r="A36" s="5">
         <v>33</v>
       </c>
-      <c r="B36" s="33" t="s">
+      <c r="B36" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="33" t="s">
+      <c r="C36" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D36" s="33" t="s">
+      <c r="D36" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E36" s="35" t="s">
+      <c r="E36" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="F36" s="33" t="s">
+      <c r="F36" s="1" t="s">
         <v>90</v>
       </c>
       <c r="G36" s="15" t="s">
@@ -3357,23 +3352,23 @@
       <c r="G40" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="H40" s="35" t="s">
+      <c r="H40" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I40" s="35"/>
-      <c r="J40" s="35" t="s">
-        <v>148</v>
-      </c>
-      <c r="K40" s="38" t="s">
+      <c r="I40" s="6"/>
+      <c r="J40" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K40" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="L40" s="35" t="s">
-        <v>148</v>
-      </c>
-      <c r="M40" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="N40" s="33" t="s">
+      <c r="L40" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N40" s="1" t="s">
         <v>148</v>
       </c>
       <c r="O40" s="7" t="s">
@@ -3396,13 +3391,13 @@
       <c r="C41" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="34">
+      <c r="D41" s="28">
         <v>46071.40525462963</v>
       </c>
-      <c r="E41" s="36" t="s">
+      <c r="E41" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="F41" s="34"/>
+      <c r="F41" s="28"/>
       <c r="G41" s="15" t="s">
         <v>141</v>
       </c>
@@ -3438,7 +3433,7 @@
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A42" s="33"/>
+      <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3450,13 +3445,13 @@
       <c r="H42" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I42" s="37" t="s">
+      <c r="I42" s="30" t="s">
         <v>39</v>
       </c>
       <c r="J42" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="K42" s="37" t="s">
+      <c r="K42" s="30" t="s">
         <v>39</v>
       </c>
       <c r="L42" s="14">
@@ -3468,10 +3463,10 @@
       <c r="N42" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="O42" s="39">
+      <c r="O42" s="31">
         <v>0.6875</v>
       </c>
-      <c r="P42" s="40" t="s">
+      <c r="P42" s="32" t="s">
         <v>193</v>
       </c>
       <c r="Q42" s="26" t="s">

</xml_diff>

<commit_message>
Diss: Final Software Version
</commit_message>
<xml_diff>
--- a/00_data/xx_column_mapping.xlsx
+++ b/00_data/xx_column_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/29cb6aa242dd6fa3/00_Documents/06_university/00_university_of_sussex/05_summer_semester/05_dissertation/00_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="853" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7802705-95DD-4D2D-BDB6-7B12640B80D0}"/>
+  <xr:revisionPtr revIDLastSave="854" documentId="13_ncr:1_{3227DB1A-CCC2-4825-85D7-8E8C74A669C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9554C7B-580C-4BFE-A17D-B60F4D32CBDA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7347838F-0C8E-4968-9B67-1760078DFEBA}"/>
   </bookViews>
@@ -1048,10 +1048,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1374,8 +1370,8 @@
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="4" width="43.77734375" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="43.77734375" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="66.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5546875" customWidth="1"/>

</xml_diff>